<commit_message>
Flipkart step 6: columns and table
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/fixtures/flipkart/flipkart-orders.xlsx
+++ b/test/fixtures/flipkart/flipkart-orders.xlsx
@@ -17,7 +17,7 @@
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="1">
+  <futureMetadata name="XLRICHVALUE" count="2">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -25,17 +25,27 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="1"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
-  <valueMetadata count="1">
+  <valueMetadata count="2">
     <bk>
       <rc t="1" v="0"/>
     </bk>
+    <bk>
+      <rc t="1" v="1"/>
+    </bk>
   </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="40">
   <si>
     <t>Order ID</t>
   </si>
@@ -70,7 +80,10 @@
     <t>Email ID</t>
   </si>
   <si>
-    <t>OD-TEST-000000000002</t>
+    <t>Review Screenshot</t>
+  </si>
+  <si>
+    <t>OD100000000000000002</t>
   </si>
   <si>
     <t>Test Brand Steel Bottle</t>
@@ -91,7 +104,10 @@
     <t>test.person2@example.test</t>
   </si>
   <si>
-    <t>OD-TEST-000000000003</t>
+    <t>https://drive.google.com/open?id=1TestFlipkartReview02abcd</t>
+  </si>
+  <si>
+    <t>OD100000000000000003</t>
   </si>
   <si>
     <t>21-07-2026</t>
@@ -115,7 +131,7 @@
     <t>test.person3@example.test</t>
   </si>
   <si>
-    <t>OD-TEST-000000000004</t>
+    <t>OD100000000000000004</t>
   </si>
   <si>
     <t>Test Person Four</t>
@@ -131,7 +147,10 @@
     <t>test.person4@example.test</t>
   </si>
   <si>
-    <t>OD-TEST-000000000006</t>
+    <t>Review screenshot</t>
+  </si>
+  <si>
+    <t>OD100000000000000006</t>
   </si>
   <si>
     <t>Test Person Six</t>
@@ -141,6 +160,9 @@
   </si>
   <si>
     <t>Not delivered yet</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1TestFlipkartReview06abcd</t>
   </si>
   <si>
     <t>Made-up notes: this tab is not read.</t>
@@ -293,9 +315,13 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
   <rv s="0">
     <v>0</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>1</v>
     <v>5</v>
   </rv>
 </rvData>
@@ -313,6 +339,7 @@
 <file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
 <richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <rel r:id="rId1"/>
+  <rel r:id="rId2"/>
 </richValueRels>
 </file>
 
@@ -671,10 +698,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
@@ -682,9 +709,10 @@
     <col min="6" max="7" width="40" customWidth="1"/>
     <col min="8" max="8" width="60" customWidth="1"/>
     <col min="9" max="9" width="26" customWidth="1"/>
+    <col min="10" max="10" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -712,113 +740,128 @@
       <c r="I1" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="J1" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2" s="2">
         <v>46223</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2">
         <v>349</v>
       </c>
       <c r="E2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I2" t="s">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="J2" t="s">
+        <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F3" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
       <c r="H3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I3" t="s">
-        <v>25</v>
+        <v>27</v>
+      </c>
+      <c r="J3" t="e" vm="2">
+        <v>#VALUE!</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B4" s="2">
         <v>46225</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D4">
         <v>349.5</v>
       </c>
       <c r="E4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H4" t="str">
         <f>HYPERLINK("https://www.flipkart.com/test-brand-steel-bottle/product-reviews/itmTEST000000004?pid=TESTPID0000004","Open review")</f>
         <v>Open review</v>
       </c>
       <c r="I4" t="s">
-        <v>30</v>
+        <v>32</v>
+      </c>
+      <c r="J4" t="s">
+        <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B6" s="2">
         <v>46226</v>
       </c>
       <c r="C6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D6">
         <v>499</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="G6" t="s">
-        <v>34</v>
+        <v>37</v>
+      </c>
+      <c r="J6" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -826,10 +869,11 @@
     <hyperlink ref="F2" r:id="rId1"/>
     <hyperlink ref="G2" r:id="rId2"/>
     <hyperlink ref="H2" r:id="rId3"/>
+    <hyperlink ref="J4" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <drawing r:id="rId4"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
 
@@ -840,7 +884,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>